<commit_message>
finalizing changes to make it perfect logged in
</commit_message>
<xml_diff>
--- a/logs/trading_report.xlsx
+++ b/logs/trading_report.xlsx
@@ -68736,7 +68736,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z10"/>
+  <dimension ref="A1:Z11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69444,6 +69444,68 @@
         <v>6400995</v>
       </c>
       <c r="Z10" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>5800800</v>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>BTCUSD</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>45906.61646990741</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>110787.3</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2025-09-06 14:48:19</t>
+        </is>
+      </c>
+      <c r="S11" t="n">
+        <v>110803.4</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="U11" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="V11" t="n">
+        <v>-1.66</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="inlineStr"/>
+      <c r="Y11" t="n">
+        <v>6428448</v>
+      </c>
+      <c r="Z11" t="inlineStr">
         <is>
           <t>2025-09</t>
         </is>
@@ -69524,19 +69586,19 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C3" t="n">
-        <v>16.02</v>
+        <v>16.18</v>
       </c>
       <c r="D3" t="n">
         <v>-519</v>
       </c>
       <c r="E3" t="n">
-        <v>-502.98</v>
+        <v>-502.82</v>
       </c>
       <c r="F3" t="n">
-        <v>4.06</v>
+        <v>4.07</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
4.0 finalize thing running part
</commit_message>
<xml_diff>
--- a/logs/trading_report.xlsx
+++ b/logs/trading_report.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ActivityLog" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TradeHistory" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlySummary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ActivityLog" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="TradeHistory" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlySummary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4523"/>
+  <dimension ref="A1:C4561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69089,6 +69089,656 @@
         </is>
       </c>
     </row>
+    <row r="4524">
+      <c r="A4524" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:06</t>
+        </is>
+      </c>
+      <c r="B4524" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C4524" t="inlineStr">
+        <is>
+          <t>MT5 initialize() failed, error code = (-10005, 'IPC timeout')</t>
+        </is>
+      </c>
+    </row>
+    <row r="4525">
+      <c r="A4525" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:08</t>
+        </is>
+      </c>
+      <c r="B4525" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C4525" t="inlineStr">
+        <is>
+          <t>An exception occurred during MT5 initialization: Failed to initialize MT5
+Traceback (most recent call last):
+  File "C:\Users\Administrator\Documents\GitHub\goldiebot-backend\trade_manager.py", line 28, in __enter__
+    raise ConnectionError("Failed to initialize MT5")
+ConnectionError: Failed to initialize MT5</t>
+        </is>
+      </c>
+    </row>
+    <row r="4526">
+      <c r="A4526" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:09</t>
+        </is>
+      </c>
+      <c r="B4526" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="C4526" t="inlineStr">
+        <is>
+          <t>Could not establish connection to MetaTrader 5. Shutting down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4527">
+      <c r="A4527" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:14</t>
+        </is>
+      </c>
+      <c r="B4527" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4527" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4528">
+      <c r="A4528" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:15</t>
+        </is>
+      </c>
+      <c r="B4528" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4528" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4529">
+      <c r="A4529" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:16</t>
+        </is>
+      </c>
+      <c r="B4529" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4529" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4530">
+      <c r="A4530" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:17</t>
+        </is>
+      </c>
+      <c r="B4530" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4530" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4531">
+      <c r="A4531" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:23</t>
+        </is>
+      </c>
+      <c r="B4531" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4531" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4532">
+      <c r="A4532" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:24</t>
+        </is>
+      </c>
+      <c r="B4532" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4532" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4533">
+      <c r="A4533" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:25</t>
+        </is>
+      </c>
+      <c r="B4533" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4533" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4534">
+      <c r="A4534" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:27</t>
+        </is>
+      </c>
+      <c r="B4534" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4534" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4535">
+      <c r="A4535" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:41:33</t>
+        </is>
+      </c>
+      <c r="B4535" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4535" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4536">
+      <c r="A4536" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:27</t>
+        </is>
+      </c>
+      <c r="B4536" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4536" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4537">
+      <c r="A4537" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:28</t>
+        </is>
+      </c>
+      <c r="B4537" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4537" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4538">
+      <c r="A4538" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:29</t>
+        </is>
+      </c>
+      <c r="B4538" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4538" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4539">
+      <c r="A4539" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:30</t>
+        </is>
+      </c>
+      <c r="B4539" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4539" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4540">
+      <c r="A4540" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:36</t>
+        </is>
+      </c>
+      <c r="B4540" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4540" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4541">
+      <c r="A4541" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:37</t>
+        </is>
+      </c>
+      <c r="B4541" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4541" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4542">
+      <c r="A4542" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:38</t>
+        </is>
+      </c>
+      <c r="B4542" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4542" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4543">
+      <c r="A4543" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:39</t>
+        </is>
+      </c>
+      <c r="B4543" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4543" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4544">
+      <c r="A4544" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:45</t>
+        </is>
+      </c>
+      <c r="B4544" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4544" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4545">
+      <c r="A4545" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:46</t>
+        </is>
+      </c>
+      <c r="B4545" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4545" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4546">
+      <c r="A4546" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:48</t>
+        </is>
+      </c>
+      <c r="B4546" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4546" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4547">
+      <c r="A4547" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:49</t>
+        </is>
+      </c>
+      <c r="B4547" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4547" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4548">
+      <c r="A4548" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:55</t>
+        </is>
+      </c>
+      <c r="B4548" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4548" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4549">
+      <c r="A4549" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:56</t>
+        </is>
+      </c>
+      <c r="B4549" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4549" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4550">
+      <c r="A4550" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:57</t>
+        </is>
+      </c>
+      <c r="B4550" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4550" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4551">
+      <c r="A4551" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:43:58</t>
+        </is>
+      </c>
+      <c r="B4551" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4551" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4552">
+      <c r="A4552" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:04</t>
+        </is>
+      </c>
+      <c r="B4552" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4552" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4553">
+      <c r="A4553" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:05</t>
+        </is>
+      </c>
+      <c r="B4553" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4553" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4554">
+      <c r="A4554" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:07</t>
+        </is>
+      </c>
+      <c r="B4554" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4554" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4555">
+      <c r="A4555" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:08</t>
+        </is>
+      </c>
+      <c r="B4555" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4555" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4556">
+      <c r="A4556" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:14</t>
+        </is>
+      </c>
+      <c r="B4556" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4556" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4557">
+      <c r="A4557" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:15</t>
+        </is>
+      </c>
+      <c r="B4557" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4557" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4558">
+      <c r="A4558" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:16</t>
+        </is>
+      </c>
+      <c r="B4558" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4558" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4559">
+      <c r="A4559" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:17</t>
+        </is>
+      </c>
+      <c r="B4559" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4559" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4560">
+      <c r="A4560" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:23</t>
+        </is>
+      </c>
+      <c r="B4560" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4560" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4561">
+      <c r="A4561" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:25</t>
+        </is>
+      </c>
+      <c r="B4561" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4561" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
done with this 4.0
</commit_message>
<xml_diff>
--- a/logs/trading_report.xlsx
+++ b/logs/trading_report.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4561"/>
+  <dimension ref="A1:C4686"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -69739,6 +69739,2131 @@
         </is>
       </c>
     </row>
+    <row r="4562">
+      <c r="A4562" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:26</t>
+        </is>
+      </c>
+      <c r="B4562" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4562" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4563">
+      <c r="A4563" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:28</t>
+        </is>
+      </c>
+      <c r="B4563" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4563" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4564">
+      <c r="A4564" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:34</t>
+        </is>
+      </c>
+      <c r="B4564" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4564" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4565">
+      <c r="A4565" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:36</t>
+        </is>
+      </c>
+      <c r="B4565" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4565" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4566">
+      <c r="A4566" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:37</t>
+        </is>
+      </c>
+      <c r="B4566" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4566" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4567">
+      <c r="A4567" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:38</t>
+        </is>
+      </c>
+      <c r="B4567" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4567" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4568">
+      <c r="A4568" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:45</t>
+        </is>
+      </c>
+      <c r="B4568" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4568" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4569">
+      <c r="A4569" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:46</t>
+        </is>
+      </c>
+      <c r="B4569" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4569" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4570">
+      <c r="A4570" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:47</t>
+        </is>
+      </c>
+      <c r="B4570" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4570" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4571">
+      <c r="A4571" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:48</t>
+        </is>
+      </c>
+      <c r="B4571" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4571" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4572">
+      <c r="A4572" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:55</t>
+        </is>
+      </c>
+      <c r="B4572" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4572" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4573">
+      <c r="A4573" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:56</t>
+        </is>
+      </c>
+      <c r="B4573" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4573" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4574">
+      <c r="A4574" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:58</t>
+        </is>
+      </c>
+      <c r="B4574" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4574" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4575">
+      <c r="A4575" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:44:59</t>
+        </is>
+      </c>
+      <c r="B4575" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4575" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4576">
+      <c r="A4576" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:05</t>
+        </is>
+      </c>
+      <c r="B4576" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4576" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4577">
+      <c r="A4577" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:07</t>
+        </is>
+      </c>
+      <c r="B4577" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4577" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4578">
+      <c r="A4578" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:08</t>
+        </is>
+      </c>
+      <c r="B4578" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4578" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4579">
+      <c r="A4579" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:10</t>
+        </is>
+      </c>
+      <c r="B4579" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4579" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4580">
+      <c r="A4580" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:16</t>
+        </is>
+      </c>
+      <c r="B4580" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4580" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4581">
+      <c r="A4581" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:18</t>
+        </is>
+      </c>
+      <c r="B4581" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4581" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4582">
+      <c r="A4582" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:19</t>
+        </is>
+      </c>
+      <c r="B4582" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4582" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4583">
+      <c r="A4583" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:21</t>
+        </is>
+      </c>
+      <c r="B4583" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4583" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4584">
+      <c r="A4584" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:27</t>
+        </is>
+      </c>
+      <c r="B4584" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4584" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4585">
+      <c r="A4585" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:28</t>
+        </is>
+      </c>
+      <c r="B4585" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4585" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4586">
+      <c r="A4586" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:30</t>
+        </is>
+      </c>
+      <c r="B4586" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4586" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4587">
+      <c r="A4587" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:31</t>
+        </is>
+      </c>
+      <c r="B4587" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4587" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4588">
+      <c r="A4588" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:38</t>
+        </is>
+      </c>
+      <c r="B4588" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4588" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4589">
+      <c r="A4589" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:39</t>
+        </is>
+      </c>
+      <c r="B4589" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4589" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4590">
+      <c r="A4590" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:40</t>
+        </is>
+      </c>
+      <c r="B4590" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4590" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4591">
+      <c r="A4591" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:42</t>
+        </is>
+      </c>
+      <c r="B4591" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4591" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4592">
+      <c r="A4592" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:48</t>
+        </is>
+      </c>
+      <c r="B4592" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4592" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4593">
+      <c r="A4593" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:50</t>
+        </is>
+      </c>
+      <c r="B4593" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4593" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4594">
+      <c r="A4594" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:51</t>
+        </is>
+      </c>
+      <c r="B4594" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4594" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4595">
+      <c r="A4595" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:52</t>
+        </is>
+      </c>
+      <c r="B4595" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4595" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4596">
+      <c r="A4596" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:45:59</t>
+        </is>
+      </c>
+      <c r="B4596" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4596" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4597">
+      <c r="A4597" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:00</t>
+        </is>
+      </c>
+      <c r="B4597" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4597" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4598">
+      <c r="A4598" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:02</t>
+        </is>
+      </c>
+      <c r="B4598" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4598" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4599">
+      <c r="A4599" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:03</t>
+        </is>
+      </c>
+      <c r="B4599" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4599" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4600">
+      <c r="A4600" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:10</t>
+        </is>
+      </c>
+      <c r="B4600" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4600" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4601">
+      <c r="A4601" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:11</t>
+        </is>
+      </c>
+      <c r="B4601" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4601" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4602">
+      <c r="A4602" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:13</t>
+        </is>
+      </c>
+      <c r="B4602" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4602" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4603">
+      <c r="A4603" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:14</t>
+        </is>
+      </c>
+      <c r="B4603" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4603" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4604">
+      <c r="A4604" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:21</t>
+        </is>
+      </c>
+      <c r="B4604" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4604" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4605">
+      <c r="A4605" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:23</t>
+        </is>
+      </c>
+      <c r="B4605" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4605" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4606">
+      <c r="A4606" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:24</t>
+        </is>
+      </c>
+      <c r="B4606" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4606" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4607">
+      <c r="A4607" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:26</t>
+        </is>
+      </c>
+      <c r="B4607" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4607" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4608">
+      <c r="A4608" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:32</t>
+        </is>
+      </c>
+      <c r="B4608" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4608" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4609">
+      <c r="A4609" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:33</t>
+        </is>
+      </c>
+      <c r="B4609" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4609" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4610">
+      <c r="A4610" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:34</t>
+        </is>
+      </c>
+      <c r="B4610" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4610" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4611">
+      <c r="A4611" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:36</t>
+        </is>
+      </c>
+      <c r="B4611" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4611" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4612">
+      <c r="A4612" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:42</t>
+        </is>
+      </c>
+      <c r="B4612" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4612" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4613">
+      <c r="A4613" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:43</t>
+        </is>
+      </c>
+      <c r="B4613" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4613" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4614">
+      <c r="A4614" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:44</t>
+        </is>
+      </c>
+      <c r="B4614" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4614" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4615">
+      <c r="A4615" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:45</t>
+        </is>
+      </c>
+      <c r="B4615" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4615" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4616">
+      <c r="A4616" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:51</t>
+        </is>
+      </c>
+      <c r="B4616" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4616" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4617">
+      <c r="A4617" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:52</t>
+        </is>
+      </c>
+      <c r="B4617" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4617" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4618">
+      <c r="A4618" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:53</t>
+        </is>
+      </c>
+      <c r="B4618" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4618" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4619">
+      <c r="A4619" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:46:54</t>
+        </is>
+      </c>
+      <c r="B4619" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4619" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4620">
+      <c r="A4620" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:02</t>
+        </is>
+      </c>
+      <c r="B4620" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4620" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4621">
+      <c r="A4621" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:03</t>
+        </is>
+      </c>
+      <c r="B4621" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4621" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4622">
+      <c r="A4622" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:05</t>
+        </is>
+      </c>
+      <c r="B4622" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4622" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4623">
+      <c r="A4623" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:07</t>
+        </is>
+      </c>
+      <c r="B4623" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4623" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4624">
+      <c r="A4624" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:13</t>
+        </is>
+      </c>
+      <c r="B4624" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4624" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4625">
+      <c r="A4625" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:15</t>
+        </is>
+      </c>
+      <c r="B4625" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4625" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4626">
+      <c r="A4626" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:16</t>
+        </is>
+      </c>
+      <c r="B4626" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4626" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4627">
+      <c r="A4627" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:17</t>
+        </is>
+      </c>
+      <c r="B4627" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4627" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4628">
+      <c r="A4628" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:24</t>
+        </is>
+      </c>
+      <c r="B4628" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4628" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4629">
+      <c r="A4629" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:25</t>
+        </is>
+      </c>
+      <c r="B4629" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4629" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4630">
+      <c r="A4630" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:26</t>
+        </is>
+      </c>
+      <c r="B4630" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4630" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4631">
+      <c r="A4631" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:27</t>
+        </is>
+      </c>
+      <c r="B4631" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4631" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4632">
+      <c r="A4632" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:33</t>
+        </is>
+      </c>
+      <c r="B4632" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4632" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4633">
+      <c r="A4633" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:34</t>
+        </is>
+      </c>
+      <c r="B4633" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4633" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4634">
+      <c r="A4634" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:35</t>
+        </is>
+      </c>
+      <c r="B4634" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4634" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4635">
+      <c r="A4635" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:37</t>
+        </is>
+      </c>
+      <c r="B4635" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4635" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4636">
+      <c r="A4636" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:43</t>
+        </is>
+      </c>
+      <c r="B4636" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4636" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4637">
+      <c r="A4637" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:44</t>
+        </is>
+      </c>
+      <c r="B4637" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4637" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4638">
+      <c r="A4638" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:45</t>
+        </is>
+      </c>
+      <c r="B4638" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4638" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4639">
+      <c r="A4639" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:46</t>
+        </is>
+      </c>
+      <c r="B4639" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4639" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4640">
+      <c r="A4640" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:52</t>
+        </is>
+      </c>
+      <c r="B4640" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4640" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4641">
+      <c r="A4641" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:53</t>
+        </is>
+      </c>
+      <c r="B4641" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4641" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4642">
+      <c r="A4642" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:54</t>
+        </is>
+      </c>
+      <c r="B4642" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4642" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4643">
+      <c r="A4643" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:47:55</t>
+        </is>
+      </c>
+      <c r="B4643" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4643" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4644">
+      <c r="A4644" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:01</t>
+        </is>
+      </c>
+      <c r="B4644" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4644" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4645">
+      <c r="A4645" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:03</t>
+        </is>
+      </c>
+      <c r="B4645" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4645" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4646">
+      <c r="A4646" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:04</t>
+        </is>
+      </c>
+      <c r="B4646" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4646" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4647">
+      <c r="A4647" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:05</t>
+        </is>
+      </c>
+      <c r="B4647" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4647" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4648">
+      <c r="A4648" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:11</t>
+        </is>
+      </c>
+      <c r="B4648" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4648" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4649">
+      <c r="A4649" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:12</t>
+        </is>
+      </c>
+      <c r="B4649" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4649" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4650">
+      <c r="A4650" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:13</t>
+        </is>
+      </c>
+      <c r="B4650" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4650" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4651">
+      <c r="A4651" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:14</t>
+        </is>
+      </c>
+      <c r="B4651" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4651" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4652">
+      <c r="A4652" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:21</t>
+        </is>
+      </c>
+      <c r="B4652" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4652" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4653">
+      <c r="A4653" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:23</t>
+        </is>
+      </c>
+      <c r="B4653" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4653" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4654">
+      <c r="A4654" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:24</t>
+        </is>
+      </c>
+      <c r="B4654" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4654" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4655">
+      <c r="A4655" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:26</t>
+        </is>
+      </c>
+      <c r="B4655" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4655" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4656">
+      <c r="A4656" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:33</t>
+        </is>
+      </c>
+      <c r="B4656" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4656" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4657">
+      <c r="A4657" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:35</t>
+        </is>
+      </c>
+      <c r="B4657" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4657" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4658">
+      <c r="A4658" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:36</t>
+        </is>
+      </c>
+      <c r="B4658" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4658" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4659">
+      <c r="A4659" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:38</t>
+        </is>
+      </c>
+      <c r="B4659" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4659" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4660">
+      <c r="A4660" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:44</t>
+        </is>
+      </c>
+      <c r="B4660" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4660" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4661">
+      <c r="A4661" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:48</t>
+        </is>
+      </c>
+      <c r="B4661" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4661" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4662">
+      <c r="A4662" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:53</t>
+        </is>
+      </c>
+      <c r="B4662" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4662" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4663">
+      <c r="A4663" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:48:56</t>
+        </is>
+      </c>
+      <c r="B4663" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4663" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4664">
+      <c r="A4664" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:07</t>
+        </is>
+      </c>
+      <c r="B4664" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4664" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4665">
+      <c r="A4665" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:09</t>
+        </is>
+      </c>
+      <c r="B4665" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4665" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4666">
+      <c r="A4666" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:11</t>
+        </is>
+      </c>
+      <c r="B4666" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4666" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4667">
+      <c r="A4667" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:13</t>
+        </is>
+      </c>
+      <c r="B4667" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4667" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4668">
+      <c r="A4668" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:19</t>
+        </is>
+      </c>
+      <c r="B4668" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4668" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4669">
+      <c r="A4669" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:20</t>
+        </is>
+      </c>
+      <c r="B4669" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4669" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4670">
+      <c r="A4670" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:22</t>
+        </is>
+      </c>
+      <c r="B4670" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4670" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4671">
+      <c r="A4671" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:24</t>
+        </is>
+      </c>
+      <c r="B4671" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4671" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4672">
+      <c r="A4672" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:31</t>
+        </is>
+      </c>
+      <c r="B4672" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4672" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4673">
+      <c r="A4673" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:32</t>
+        </is>
+      </c>
+      <c r="B4673" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4673" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4674">
+      <c r="A4674" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:33</t>
+        </is>
+      </c>
+      <c r="B4674" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4674" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4675">
+      <c r="A4675" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:34</t>
+        </is>
+      </c>
+      <c r="B4675" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4675" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4676">
+      <c r="A4676" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:40</t>
+        </is>
+      </c>
+      <c r="B4676" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4676" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4677">
+      <c r="A4677" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:41</t>
+        </is>
+      </c>
+      <c r="B4677" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4677" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4678">
+      <c r="A4678" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:42</t>
+        </is>
+      </c>
+      <c r="B4678" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4678" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4679">
+      <c r="A4679" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:49</t>
+        </is>
+      </c>
+      <c r="B4679" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4679" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4680">
+      <c r="A4680" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:50</t>
+        </is>
+      </c>
+      <c r="B4680" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4680" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4681">
+      <c r="A4681" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:51</t>
+        </is>
+      </c>
+      <c r="B4681" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4681" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4682">
+      <c r="A4682" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:52</t>
+        </is>
+      </c>
+      <c r="B4682" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4682" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4683">
+      <c r="A4683" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:58</t>
+        </is>
+      </c>
+      <c r="B4683" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4683" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4684">
+      <c r="A4684" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:49:59</t>
+        </is>
+      </c>
+      <c r="B4684" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4684" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4685">
+      <c r="A4685" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:50:00</t>
+        </is>
+      </c>
+      <c r="B4685" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4685" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4686">
+      <c r="A4686" t="inlineStr">
+        <is>
+          <t>2025-09-11 12:50:02</t>
+        </is>
+      </c>
+      <c r="B4686" t="inlineStr">
+        <is>
+          <t>WARNING</t>
+        </is>
+      </c>
+      <c r="C4686" t="inlineStr">
+        <is>
+          <t>positions_get() returned None. Possible connection issue.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>